<commit_message>
Fix Northlake Q4 billing mismatch and register future-date exceptions
- Correct Q4_2025_billing_export.xlsx Northlake Bioinstruments Dec
  2025 billed value from 11050 to 9350 to match ERPNext Sales
  Invoice/Sales Order Item source records, and recalculate the Q4
  total from 27660 to 25960 (formula cached values updated too).
- Add Facts and Traps.csv registering the 361 post-2026-01-12 date
  cells across Contract, Sales Order(Item), Opportunity, Prospect
  Opportunity, Email Campaign, Fiscal Year, Project, Purchase
  Invoice, Quotation, Subscription, and Task as intentional
  future-dated business commitments/forecasts rather than data
  errors, with per-file rationale.
</commit_message>
<xml_diff>
--- a/filesystem/Finance/Billing/Q4_2025_billing_export.xlsx
+++ b/filesystem/Finance/Billing/Q4_2025_billing_export.xlsx
@@ -1944,10 +1944,10 @@
         <v>8470</v>
       </c>
       <c r="E33" s="36" t="n">
-        <v>11050</v>
+        <v>9350</v>
       </c>
       <c r="F33" s="37" t="n">
-        <v>27660</v>
+        <v>25960</v>
       </c>
       <c r="G33" s="38" t="n">
         <v>3</v>
@@ -2331,11 +2331,11 @@
       </c>
       <c r="E45" s="47">
         <f>SUM(E5:E44)</f>
-        <v>548184</v>
+        <v>546484</v>
       </c>
       <c r="F45" s="47">
         <f>SUM(F5:F44)</f>
-        <v>1593900</v>
+        <v>1592200</v>
       </c>
       <c r="G45" s="48">
         <f>SUM(G5:G44)</f>

</xml_diff>